<commit_message>
fix: Lender pro forma uses year-by-year grade-band revenue + schema codegen
1. Lender pro forma now computes ESA revenue per year using actual
   grade-band enrollment × per-pupil rates (with ADA adjustment),
   instead of approximating via per-student Y1 + growth rate.
   This fixes inaccurate Y3-Y5 projections when grade mix shifts.

2. Added openingBalances, sourcesAndUses, scenarios, covenantThresholds
   to ModelFormData in openapi.yaml. Re-ran codegen so these fields
   are no longer stripped on save.

3. Added lender-specific QA assertions for Charter ADA Grade-Band:
   - Charter Funding Details section present in Assumptions
   - Per-pupil rates populated for K-5, 6-8, 9-12
   - Year-by-year grade-band revenue positive for all 5 years

All 20/20 QA tests pass. Both builds succeed.
</commit_message>
<xml_diff>
--- a/artifacts/api-server/qa-output/Lender_Pro_Forma_Charter_ADA_Grade-Band.xlsx
+++ b/artifacts/api-server/qa-output/Lender_Pro_Forma_Charter_ADA_Grade-Band.xlsx
@@ -513,7 +513,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -538,6 +538,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE8F5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF8E1"/>
       </patternFill>
     </fill>
   </fills>
@@ -601,7 +606,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -656,6 +661,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="167" fontId="13" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="13" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="165" fontId="13" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1252,7 +1260,7 @@
         <v>30</v>
       </c>
       <c r="D22" s="12">
-        <v>9925</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="3:4" x14ac:dyDescent="0.25">
@@ -1260,7 +1268,7 @@
         <v>31</v>
       </c>
       <c r="D23" s="13">
-        <v>0.005163727959697733</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="3:4" x14ac:dyDescent="0.25">
@@ -1768,15 +1776,15 @@
       </c>
       <c r="E7" s="21">
         <f>Assumptions!D14*Assumptions!D22*(1+Assumptions!D23)^2</f>
-        <v>3008329.39231738</v>
+        <v>3043400</v>
       </c>
       <c r="F7" s="21">
         <f>Assumptions!D15*Assumptions!D22*(1+Assumptions!D23)^3</f>
-        <v>4031818.11588329</v>
+        <v>4113050</v>
       </c>
       <c r="G7" s="21">
         <f>Assumptions!D16*Assumptions!D22*(1+Assumptions!D23)^4</f>
-        <v>5065796.65977087</v>
+        <v>5234700</v>
       </c>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.25">
@@ -1843,15 +1851,15 @@
       </c>
       <c r="E10" s="23">
         <f>E6+E7+E8+E9</f>
-        <v>3310637.39231738</v>
+        <v>3345708</v>
       </c>
       <c r="F10" s="23">
         <f>F6+F7+F8+F9</f>
-        <v>4381654.43588329</v>
+        <v>4462886.32</v>
       </c>
       <c r="G10" s="23">
         <f>G6+G7+G8+G9</f>
-        <v>5465898.42177087</v>
+        <v>5634801.762</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.25">
@@ -2222,15 +2230,15 @@
       </c>
       <c r="E7" s="21">
         <f>Drivers!E7</f>
-        <v>3008329.39231738</v>
+        <v>3043400</v>
       </c>
       <c r="F7" s="21">
         <f>Drivers!F7</f>
-        <v>4031818.11588329</v>
+        <v>4113050</v>
       </c>
       <c r="G7" s="21">
         <f>Drivers!G7</f>
-        <v>5065796.65977087</v>
+        <v>5234700</v>
       </c>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.25">
@@ -2297,15 +2305,15 @@
       </c>
       <c r="E10" s="23">
         <f>Drivers!E10</f>
-        <v>3310637.39231738</v>
+        <v>3345708</v>
       </c>
       <c r="F10" s="23">
         <f>Drivers!F10</f>
-        <v>4381654.43588329</v>
+        <v>4462886.32</v>
       </c>
       <c r="G10" s="23">
         <f>Drivers!G10</f>
-        <v>5465898.42177087</v>
+        <v>5634801.762</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.25">
@@ -2397,15 +2405,15 @@
       </c>
       <c r="E16" s="25">
         <f>E10-E15</f>
-        <v>73284.20199184</v>
+        <v>108354.80967446</v>
       </c>
       <c r="F16" s="24">
         <f>F10-F15</f>
-        <v>-321056.9518978</v>
+        <v>-239825.06778109</v>
       </c>
       <c r="G16" s="24">
         <f>G10-G15</f>
-        <v>-1684638.46844119</v>
+        <v>-1515735.12821206</v>
       </c>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.25">
@@ -2422,15 +2430,15 @@
       </c>
       <c r="E17" s="26">
         <f>IF(E10&gt;0,E16/E10,0)</f>
-        <v>0.02213598</v>
+        <v>0.03238621</v>
       </c>
       <c r="F17" s="26">
         <f>IF(F10&gt;0,F16/F10,0)</f>
-        <v>-0.073273</v>
+        <v>-0.05373766</v>
       </c>
       <c r="G17" s="26">
         <f>IF(G10&gt;0,G16/G10,0)</f>
-        <v>-0.30820889</v>
+        <v>-0.26899529</v>
       </c>
     </row>
   </sheetData>
@@ -2501,15 +2509,15 @@
       </c>
       <c r="E4" s="21">
         <f>'5-Year P&amp;L'!E16</f>
-        <v>73284.20199184</v>
+        <v>108354.80967446</v>
       </c>
       <c r="F4" s="21">
         <f>'5-Year P&amp;L'!F16</f>
-        <v>-321056.9518978</v>
+        <v>-239825.06778109</v>
       </c>
       <c r="G4" s="21">
         <f>'5-Year P&amp;L'!G16</f>
-        <v>-1684638.46844119</v>
+        <v>-1515735.12821206</v>
       </c>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.25">
@@ -2599,17 +2607,17 @@
         <f>IF(D8&gt;0,D4/D8,IF(D4&gt;0,99.9,0))</f>
         <v>0.35643157</v>
       </c>
-      <c r="E10" s="27">
+      <c r="E10" s="28">
         <f>IF(E8&gt;0,E4/E8,IF(E4&gt;0,99.9,0))</f>
-        <v>0.6872846</v>
+        <v>1.01618889</v>
       </c>
       <c r="F10" s="27">
         <f>IF(F8&gt;0,F4/F8,IF(F4&gt;0,99.9,0))</f>
-        <v>-3.01098316</v>
+        <v>-2.24916245</v>
       </c>
       <c r="G10" s="27">
         <f>IF(G8&gt;0,G4/G8,IF(G4&gt;0,99.9,0))</f>
-        <v>-15.79912235</v>
+        <v>-14.2150884</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.25">
@@ -2626,40 +2634,40 @@
       </c>
       <c r="E12" s="21">
         <f>E4-E8</f>
-        <v>-33344.40882365</v>
+        <v>1726.19885897</v>
       </c>
       <c r="F12" s="21">
         <f>F4-F8</f>
-        <v>-427685.56271329</v>
+        <v>-346453.67859658</v>
       </c>
       <c r="G12" s="21">
         <f>G4-G8</f>
-        <v>-1791267.07925669</v>
+        <v>-1622363.73902756</v>
       </c>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B14" s="22" t="s">
         <v>119</v>
       </c>
-      <c r="C14" s="28">
+      <c r="C14" s="29">
         <f>Assumptions!D57+C12</f>
         <v>-282114.89652978</v>
       </c>
-      <c r="D14" s="28">
+      <c r="D14" s="29">
         <f>C14+D12</f>
         <v>-350737.70382146</v>
       </c>
-      <c r="E14" s="28">
+      <c r="E14" s="29">
         <f>D14+E12</f>
-        <v>-384082.11264511</v>
-      </c>
-      <c r="F14" s="28">
+        <v>-349011.50496249</v>
+      </c>
+      <c r="F14" s="29">
         <f>E14+F12</f>
-        <v>-811767.6753584</v>
-      </c>
-      <c r="G14" s="28">
+        <v>-695465.18355908</v>
+      </c>
+      <c r="G14" s="29">
         <f>F14+G12</f>
-        <v>-2603034.75461509</v>
+        <v>-2317828.92258663</v>
       </c>
     </row>
   </sheetData>
@@ -2770,23 +2778,23 @@
       <c r="B6" s="22" t="s">
         <v>123</v>
       </c>
-      <c r="C6" s="29">
+      <c r="C6" s="30">
         <f>C4+C5</f>
         <v>15</v>
       </c>
-      <c r="D6" s="29">
+      <c r="D6" s="30">
         <f>D4+D5</f>
         <v>21</v>
       </c>
-      <c r="E6" s="29">
+      <c r="E6" s="30">
         <f>E4+E5</f>
         <v>29</v>
       </c>
-      <c r="F6" s="29">
+      <c r="F6" s="30">
         <f>F4+F5</f>
         <v>36</v>
       </c>
-      <c r="G6" s="29">
+      <c r="G6" s="30">
         <f>G4+G5</f>
         <v>44</v>
       </c>
@@ -2854,7 +2862,7 @@
       <c r="B6" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="C6" s="30">
+      <c r="C6" s="31">
         <f>IF(Assumptions!D59&gt;0,PMT(Assumptions!D60/12,Assumptions!D61*12,-Assumptions!D59)*12,0)</f>
         <v>46628.61081549</v>
       </c>
@@ -2951,16 +2959,16 @@
       </c>
       <c r="C9" s="21">
         <f>Drivers!G10</f>
-        <v>5465898.42177087</v>
+        <v>5634801.762</v>
       </c>
     </row>
     <row r="10" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B10" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="C10" s="28">
+      <c r="C10" s="29">
         <f>'5-Year P&amp;L'!G16</f>
-        <v>-1684638.46844119</v>
+        <v>-1515735.12821206</v>
       </c>
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
fix: Lender pro forma uses year-by-year grade-band revenue (no formula collapse)
1. Lender pro forma now computes ESA revenue per year using actual
   grade-band enrollment × per-pupil rates (with ADA adjustment),
   instead of approximating via per-student Y1 + growth rate.

2. Drivers sheet writes hard values (not formulas) for ESA revenue
   when grade-band is active, preventing formula collapse to $0
   when Excel recalculates (since D22/D23 are intentionally 0).

3. Added openingBalances, sourcesAndUses, scenarios, covenantThresholds
   to ModelFormData in openapi.yaml + re-ran codegen.

4. Added lender-specific QA assertions for Charter ADA Grade-Band:
   - Charter Funding Details section present in Assumptions
   - Per-pupil rates populated for K-5, 6-8, 9-12
   - Year-by-year grade-band revenue positive for all 5 years

All 20/20 QA tests pass. Both builds succeed.
</commit_message>
<xml_diff>
--- a/artifacts/api-server/qa-output/Lender_Pro_Forma_Charter_ADA_Grade-Band.xlsx
+++ b/artifacts/api-server/qa-output/Lender_Pro_Forma_Charter_ADA_Grade-Band.xlsx
@@ -1767,23 +1767,18 @@
         <v>91</v>
       </c>
       <c r="C7" s="21">
-        <f>Assumptions!D12*Assumptions!D22</f>
         <v>1191000</v>
       </c>
       <c r="D7" s="21">
-        <f>Assumptions!D13*Assumptions!D22*(1+Assumptions!D23)^1</f>
         <v>1995250</v>
       </c>
       <c r="E7" s="21">
-        <f>Assumptions!D14*Assumptions!D22*(1+Assumptions!D23)^2</f>
         <v>3043400</v>
       </c>
       <c r="F7" s="21">
-        <f>Assumptions!D15*Assumptions!D22*(1+Assumptions!D23)^3</f>
         <v>4113050</v>
       </c>
       <c r="G7" s="21">
-        <f>Assumptions!D16*Assumptions!D22*(1+Assumptions!D23)^4</f>
         <v>5234700</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update school profile entity type and file sizes for accurate data reporting
Modify `SchoolProfile` interface to include `entityType`. Adjust file sizes in `qa-report.json` and update `mapModelToTemplateInput` function in `lender-proforma-export.ts`.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: a1e7a024-8deb-4e05-bb93-350fde674463
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 792ee06b-ddea-4a5f-bc4a-56a48380c880
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/27fdbaf7-67db-442f-83d4-bebcb570d0b5/a1e7a024-8deb-4e05-bb93-350fde674463/eaAMgMc
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/api-server/qa-output/Lender_Pro_Forma_Charter_ADA_Grade-Band.xlsx
+++ b/artifacts/api-server/qa-output/Lender_Pro_Forma_Charter_ADA_Grade-Band.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="209">
   <si>
     <t>How to Use This Workbook</t>
   </si>
@@ -28,118 +28,121 @@
     <t>Heritage Academy Charter</t>
   </si>
   <si>
+    <t>Generated March 26, 2026 · nonprofit_501c3</t>
+  </si>
+  <si>
+    <t>Cell Color Legend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Blue cells are editable inputs — change these to update your model.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  White cells contain formulas — do not edit (they recalculate automatically).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Green cells are key outputs and summary metrics.</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Navigation</t>
+  </si>
+  <si>
+    <t>The Assumptions tab is the central control panel — all other tabs reference it.</t>
+  </si>
+  <si>
+    <t>Structure</t>
+  </si>
+  <si>
+    <t>Assumptions &amp; Drivers: Model inputs and calculations</t>
+  </si>
+  <si>
+    <t>5-Year P&amp;L &amp; Cash Flow: Financial projections</t>
+  </si>
+  <si>
+    <t>Staffing &amp; Loan Snapshot: Personnel and debt detail</t>
+  </si>
+  <si>
+    <t>Summary &amp; Financial Health: Key metrics dashboard</t>
+  </si>
+  <si>
+    <t>Debt Service Convention</t>
+  </si>
+  <si>
+    <t>operating expense on the Operating Statement. This is a standard</t>
+  </si>
+  <si>
+    <t>simplification used in school financial underwriting that ensures internal</t>
+  </si>
+  <si>
+    <t>consistency across all tabs.</t>
+  </si>
+  <si>
+    <t>Tips</t>
+  </si>
+  <si>
+    <t>Check the Financial Health dashboard for an at-a-glance assessment.</t>
+  </si>
+  <si>
+    <t>Review key metrics: net margin, cash runway, and DSCR.</t>
+  </si>
+  <si>
+    <t>Next Steps</t>
+  </si>
+  <si>
+    <t>2. Verify enrollment and revenue projections match your plan.</t>
+  </si>
+  <si>
+    <t>3. Check the Financial Health dashboard for risk signals.</t>
+  </si>
+  <si>
+    <t>4. Share this workbook with your lender or financial advisor.</t>
+  </si>
+  <si>
+    <t>5. Update inputs as your school's plan evolves.</t>
+  </si>
+  <si>
+    <t>Disclaimer</t>
+  </si>
+  <si>
+    <t>a loan commitment, or a guarantee of funding. All projections are based on</t>
+  </si>
+  <si>
+    <t>user-provided assumptions and should be independently verified.</t>
+  </si>
+  <si>
+    <t>SCHOOLSTACK BUDGET</t>
+  </si>
+  <si>
+    <t>Lender-Ready Pro Forma</t>
+  </si>
+  <si>
+    <t>TABLE OF CONTENTS</t>
+  </si>
+  <si>
+    <t>Assumptions</t>
+  </si>
+  <si>
+    <t>Drivers</t>
+  </si>
+  <si>
+    <t>5-Year P&amp;L</t>
+  </si>
+  <si>
+    <t>Cash Flow &amp; DSCR</t>
+  </si>
+  <si>
+    <t>Staffing</t>
+  </si>
+  <si>
+    <t>Loan Snapshot</t>
+  </si>
+  <si>
+    <t>Summary</t>
+  </si>
+  <si>
     <t>Generated March 26, 2026</t>
-  </si>
-  <si>
-    <t>Cell Color Legend</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Blue cells are editable inputs — change these to update your model.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  White cells contain formulas — do not edit (they recalculate automatically).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Green cells are key outputs and summary metrics.</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Navigation</t>
-  </si>
-  <si>
-    <t>The Assumptions tab is the central control panel — all other tabs reference it.</t>
-  </si>
-  <si>
-    <t>Structure</t>
-  </si>
-  <si>
-    <t>Assumptions &amp; Drivers: Model inputs and calculations</t>
-  </si>
-  <si>
-    <t>5-Year P&amp;L &amp; Cash Flow: Financial projections</t>
-  </si>
-  <si>
-    <t>Staffing &amp; Loan Snapshot: Personnel and debt detail</t>
-  </si>
-  <si>
-    <t>Summary &amp; Financial Health: Key metrics dashboard</t>
-  </si>
-  <si>
-    <t>Debt Service Convention</t>
-  </si>
-  <si>
-    <t>operating expense on the Operating Statement. This is a standard</t>
-  </si>
-  <si>
-    <t>simplification used in school financial underwriting that ensures internal</t>
-  </si>
-  <si>
-    <t>consistency across all tabs.</t>
-  </si>
-  <si>
-    <t>Tips</t>
-  </si>
-  <si>
-    <t>Check the Financial Health dashboard for an at-a-glance assessment.</t>
-  </si>
-  <si>
-    <t>Review key metrics: net margin, cash runway, and DSCR.</t>
-  </si>
-  <si>
-    <t>Next Steps</t>
-  </si>
-  <si>
-    <t>2. Verify enrollment and revenue projections match your plan.</t>
-  </si>
-  <si>
-    <t>3. Check the Financial Health dashboard for risk signals.</t>
-  </si>
-  <si>
-    <t>4. Share this workbook with your lender or financial advisor.</t>
-  </si>
-  <si>
-    <t>5. Update inputs as your school's plan evolves.</t>
-  </si>
-  <si>
-    <t>Disclaimer</t>
-  </si>
-  <si>
-    <t>a loan commitment, or a guarantee of funding. All projections are based on</t>
-  </si>
-  <si>
-    <t>user-provided assumptions and should be independently verified.</t>
-  </si>
-  <si>
-    <t>SCHOOLSTACK BUDGET</t>
-  </si>
-  <si>
-    <t>Lender-Ready Pro Forma</t>
-  </si>
-  <si>
-    <t>TABLE OF CONTENTS</t>
-  </si>
-  <si>
-    <t>Assumptions</t>
-  </si>
-  <si>
-    <t>Drivers</t>
-  </si>
-  <si>
-    <t>5-Year P&amp;L</t>
-  </si>
-  <si>
-    <t>Cash Flow &amp; DSCR</t>
-  </si>
-  <si>
-    <t>Staffing</t>
-  </si>
-  <si>
-    <t>Loan Snapshot</t>
-  </si>
-  <si>
-    <t>Summary</t>
   </si>
   <si>
     <t>Generated by SchoolStack Budget  •  budget.schoolstack.ai</t>
@@ -1683,7 +1686,7 @@
   <sheetData>
     <row r="2" ht="30" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -1693,7 +1696,7 @@
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3" s="12" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
@@ -1703,27 +1706,27 @@
     </row>
     <row r="5" ht="24" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" s="40" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C5" s="41" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D5" s="41" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E5" s="41" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F5" s="41" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G5" s="41" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" s="27" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C6" s="28">
         <v>120</v>
@@ -1743,7 +1746,7 @@
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B7" s="27" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C7" s="29">
         <v>1414000</v>
@@ -1763,7 +1766,7 @@
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B8" s="27" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C8" s="29">
         <v>985486.2857142857</v>
@@ -1783,7 +1786,7 @@
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B9" s="27" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C9" s="29">
         <v>604000</v>
@@ -1803,7 +1806,7 @@
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B10" s="27" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C10" s="29">
         <v>106628.6108154935</v>
@@ -1823,7 +1826,7 @@
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B11" s="30" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C11" s="32">
         <v>-282114.8965297792</v>
@@ -1843,7 +1846,7 @@
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B12" s="30" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C12" s="32">
         <v>-282114.8965297792</v>
@@ -1863,7 +1866,7 @@
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B13" s="30" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C13" s="42">
         <v>-0.19951548552318188</v>
@@ -1883,7 +1886,7 @@
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B14" s="30" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C14" s="29">
         <v>11783.333333333334</v>
@@ -1903,7 +1906,7 @@
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B15" s="30" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C15" s="42">
         <v>0.6969492826833703</v>
@@ -1923,7 +1926,7 @@
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B16" s="30" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C16" s="44">
         <v>0.12814710042432814</v>
@@ -1943,7 +1946,7 @@
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="30" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C17" s="42">
         <v>-0.12410628409779752</v>
@@ -1963,7 +1966,7 @@
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" s="30" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C18" s="45">
         <v>-1.645771096258031</v>
@@ -1983,10 +1986,10 @@
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B19" s="30" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C19" s="47" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D19" s="47"/>
       <c r="E19" s="47"/>
@@ -1995,10 +1998,10 @@
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B20" s="30" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C20" s="48" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D20" s="48"/>
       <c r="E20" s="48"/>
@@ -2007,129 +2010,129 @@
     </row>
     <row r="22" ht="24" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B22" s="40" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C22" s="40" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D22" s="40" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E22" s="40"/>
       <c r="F22" s="40" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G22" s="40"/>
     </row>
     <row r="23" ht="45" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B23" s="49" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C23" s="50" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D23" s="51" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E23" s="51"/>
       <c r="F23" s="52" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="G23" s="52"/>
     </row>
     <row r="24" ht="45" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B24" s="49" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C24" s="50" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D24" s="51" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="E24" s="51"/>
       <c r="F24" s="52" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="G24" s="52"/>
     </row>
     <row r="25" ht="45" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B25" s="49" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C25" s="53" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D25" s="51" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E25" s="51"/>
       <c r="F25" s="52" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="G25" s="52"/>
     </row>
     <row r="26" ht="45" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B26" s="49" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C26" s="50" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D26" s="51" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E26" s="51"/>
       <c r="F26" s="52" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="G26" s="52"/>
     </row>
     <row r="27" ht="45" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B27" s="49" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C27" s="50" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D27" s="51" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E27" s="51"/>
       <c r="F27" s="52" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="G27" s="52"/>
     </row>
     <row r="28" ht="45" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B28" s="49" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C28" s="53" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D28" s="51" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E28" s="51"/>
       <c r="F28" s="52" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="G28" s="52"/>
     </row>
     <row r="29" ht="45" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B29" s="49" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C29" s="50" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D29" s="51" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E29" s="51"/>
       <c r="F29" s="52" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="G29" s="52"/>
     </row>
@@ -2138,14 +2141,14 @@
         <v>39</v>
       </c>
       <c r="C31" s="30" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D31" s="30"/>
       <c r="E31" s="30"/>
     </row>
     <row r="33" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B33" s="54" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C33" s="54"/>
       <c r="D33" s="54"/>
@@ -2339,13 +2342,13 @@
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B18" s="12" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="C18" s="12"/>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B19" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C19" s="12"/>
     </row>
@@ -2392,7 +2395,7 @@
   <sheetData>
     <row r="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B1" s="13" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C1" s="13"/>
       <c r="D1" s="13"/>
@@ -2402,19 +2405,19 @@
         <v>7</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" s="16" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C3" s="16"/>
       <c r="D3" s="16"/>
     </row>
     <row r="5" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C5" s="17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D5" s="18" t="s">
         <v>1</v>
@@ -2422,23 +2425,23 @@
     </row>
     <row r="6" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C6" s="17" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C7" s="17" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C8" s="17" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D8" s="18">
         <v>2026</v>
@@ -2446,14 +2449,14 @@
     </row>
     <row r="10" ht="24" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B10" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C10" s="16"/>
       <c r="D10" s="16"/>
     </row>
     <row r="12" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C12" s="17" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D12" s="19">
         <v>120</v>
@@ -2461,7 +2464,7 @@
     </row>
     <row r="13" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C13" s="17" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D13" s="19">
         <v>200</v>
@@ -2469,7 +2472,7 @@
     </row>
     <row r="14" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C14" s="17" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D14" s="19">
         <v>300</v>
@@ -2477,7 +2480,7 @@
     </row>
     <row r="15" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C15" s="17" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D15" s="19">
         <v>400</v>
@@ -2485,7 +2488,7 @@
     </row>
     <row r="16" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C16" s="17" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D16" s="19">
         <v>500</v>
@@ -2493,14 +2496,14 @@
     </row>
     <row r="18" ht="24" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B18" s="16" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C18" s="16"/>
       <c r="D18" s="16"/>
     </row>
     <row r="20" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C20" s="17" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D20" s="20">
         <v>0</v>
@@ -2508,7 +2511,7 @@
     </row>
     <row r="21" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C21" s="17" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D21" s="21">
         <v>0.03</v>
@@ -2516,7 +2519,7 @@
     </row>
     <row r="22" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C22" s="17" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D22" s="20">
         <v>0</v>
@@ -2524,7 +2527,7 @@
     </row>
     <row r="23" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C23" s="17" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D23" s="21">
         <v>0</v>
@@ -2532,7 +2535,7 @@
     </row>
     <row r="24" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C24" s="17" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D24" s="20">
         <v>400</v>
@@ -2540,7 +2543,7 @@
     </row>
     <row r="25" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C25" s="17" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D25" s="21">
         <v>0.03</v>
@@ -2548,7 +2551,7 @@
     </row>
     <row r="26" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C26" s="17" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D26" s="21">
         <v>0.95</v>
@@ -2556,7 +2559,7 @@
     </row>
     <row r="27" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C27" s="17" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D27" s="20">
         <v>175000</v>
@@ -2564,7 +2567,7 @@
     </row>
     <row r="28" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C28" s="17" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D28" s="21">
         <v>0</v>
@@ -2572,14 +2575,14 @@
     </row>
     <row r="30" ht="24" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B30" s="16" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C30" s="16"/>
       <c r="D30" s="16"/>
     </row>
     <row r="32" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C32" s="17" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D32" s="19">
         <v>13</v>
@@ -2587,7 +2590,7 @@
     </row>
     <row r="33" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C33" s="17" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D33" s="20">
         <v>43667</v>
@@ -2595,7 +2598,7 @@
     </row>
     <row r="34" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C34" s="17" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D34" s="21">
         <v>0.03</v>
@@ -2603,7 +2606,7 @@
     </row>
     <row r="35" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C35" s="17" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D35" s="19">
         <v>5</v>
@@ -2611,7 +2614,7 @@
     </row>
     <row r="36" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C36" s="17" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D36" s="19">
         <v>5</v>
@@ -2619,7 +2622,7 @@
     </row>
     <row r="37" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C37" s="17" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D37" s="19">
         <v>5</v>
@@ -2627,7 +2630,7 @@
     </row>
     <row r="38" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C38" s="17" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D38" s="19">
         <v>5</v>
@@ -2635,7 +2638,7 @@
     </row>
     <row r="39" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C39" s="17" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D39" s="19">
         <v>5</v>
@@ -2643,7 +2646,7 @@
     </row>
     <row r="40" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C40" s="17" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D40" s="20">
         <v>71250</v>
@@ -2651,7 +2654,7 @@
     </row>
     <row r="41" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C41" s="17" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D41" s="21">
         <v>0.03</v>
@@ -2659,7 +2662,7 @@
     </row>
     <row r="42" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C42" s="17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D42" s="21">
         <v>0.24285714285714285</v>
@@ -2667,14 +2670,14 @@
     </row>
     <row r="44" ht="24" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B44" s="16" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C44" s="16"/>
       <c r="D44" s="16"/>
     </row>
     <row r="46" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C46" s="17" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D46" s="20">
         <v>322000</v>
@@ -2682,7 +2685,7 @@
     </row>
     <row r="47" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C47" s="17" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D47" s="21">
         <v>0.03</v>
@@ -2690,7 +2693,7 @@
     </row>
     <row r="48" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C48" s="17" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D48" s="20">
         <v>0</v>
@@ -2698,7 +2701,7 @@
     </row>
     <row r="49" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C49" s="17" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D49" s="21">
         <v>0.03</v>
@@ -2706,7 +2709,7 @@
     </row>
     <row r="50" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C50" s="17" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D50" s="20">
         <v>650</v>
@@ -2714,7 +2717,7 @@
     </row>
     <row r="51" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C51" s="17" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D51" s="21">
         <v>0.717948717948718</v>
@@ -2722,7 +2725,7 @@
     </row>
     <row r="52" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C52" s="17" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D52" s="20">
         <v>204000</v>
@@ -2730,7 +2733,7 @@
     </row>
     <row r="53" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C53" s="17" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D53" s="21">
         <v>0.515686274509804</v>
@@ -2738,14 +2741,14 @@
     </row>
     <row r="55" ht="24" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B55" s="16" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C55" s="16"/>
       <c r="D55" s="16"/>
     </row>
     <row r="57" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C57" s="17" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D57" s="20">
         <v>0</v>
@@ -2753,7 +2756,7 @@
     </row>
     <row r="58" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C58" s="17" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D58" s="20">
         <v>60000</v>
@@ -2761,7 +2764,7 @@
     </row>
     <row r="59" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C59" s="17" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D59" s="20">
         <v>350000</v>
@@ -2769,7 +2772,7 @@
     </row>
     <row r="60" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C60" s="17" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D60" s="21">
         <v>0.06</v>
@@ -2777,7 +2780,7 @@
     </row>
     <row r="61" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C61" s="17" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D61" s="19">
         <v>10</v>
@@ -2785,30 +2788,30 @@
     </row>
     <row r="64" ht="24" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B64" s="16" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C64" s="16"/>
       <c r="D64" s="16"/>
     </row>
     <row r="66" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C66" s="17" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D66" s="18" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="67" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C67" s="17" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D67" s="18" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="68" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C68" s="17" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D68" s="19">
         <v>0</v>
@@ -2816,7 +2819,7 @@
     </row>
     <row r="69" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C69" s="17" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D69" s="19">
         <v>0</v>
@@ -2824,7 +2827,7 @@
     </row>
     <row r="70" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C70" s="17" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D70" s="22">
         <v>0.95</v>
@@ -2832,7 +2835,7 @@
     </row>
     <row r="71" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C71" s="17" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D71" s="20">
         <v>8200</v>
@@ -2840,7 +2843,7 @@
     </row>
     <row r="72" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C72" s="17" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D72" s="20">
         <v>9100</v>
@@ -2848,7 +2851,7 @@
     </row>
     <row r="73" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C73" s="17" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D73" s="20">
         <v>10500</v>
@@ -2856,32 +2859,32 @@
     </row>
     <row r="75" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C75" s="23" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D75" s="23"/>
     </row>
     <row r="76" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C76" s="17" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D76" s="24" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="77" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C77" s="17" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D77" s="24" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="78" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C78" s="17" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D78" s="24" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -2920,7 +2923,7 @@
   <sheetData>
     <row r="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B1" s="13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C1" s="13"/>
       <c r="D1" s="13"/>
@@ -2931,24 +2934,24 @@
     <row r="3" ht="24" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3" s="25"/>
       <c r="C3" s="26" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D3" s="26" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E3" s="26" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F3" s="26" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G3" s="26" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B4" s="27" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C4" s="28">
         <f>Assumptions!D12</f>
@@ -2973,7 +2976,7 @@
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" s="27" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C5" s="29" t="str">
         <f>Assumptions!D12*Assumptions!D20</f>
@@ -2998,7 +3001,7 @@
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" s="27" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C6" s="29" t="str">
         <f>C5*Assumptions!D26</f>
@@ -3023,7 +3026,7 @@
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B7" s="27" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C7" s="29">
         <v>1191000</v>
@@ -3043,7 +3046,7 @@
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B8" s="27" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C8" s="29">
         <f>Assumptions!D12*Assumptions!D24</f>
@@ -3068,7 +3071,7 @@
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B9" s="27" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C9" s="29">
         <f>Assumptions!D27</f>
@@ -3093,7 +3096,7 @@
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B10" s="30" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C10" s="31">
         <f>C6+C7+C8+C9</f>
@@ -3118,7 +3121,7 @@
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B12" s="27" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C12" s="28">
         <f>CEILING(Assumptions!D12/Assumptions!D32,1)</f>
@@ -3143,7 +3146,7 @@
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B13" s="27" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C13" s="29">
         <f>C12*Assumptions!D33</f>
@@ -3168,7 +3171,7 @@
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B14" s="27" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C14" s="29">
         <f>Assumptions!D35*Assumptions!D40</f>
@@ -3193,7 +3196,7 @@
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B15" s="27" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C15" s="29">
         <f>(C13+C14)*Assumptions!D42</f>
@@ -3218,7 +3221,7 @@
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B16" s="30" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C16" s="31">
         <f>C13+C14+C15</f>
@@ -3243,7 +3246,7 @@
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" s="27" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C18" s="29">
         <f>Assumptions!D46</f>
@@ -3268,7 +3271,7 @@
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B19" s="27" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C19" s="29" t="str">
         <f>Assumptions!D48</f>
@@ -3293,7 +3296,7 @@
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B20" s="27" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C20" s="29">
         <f>Assumptions!D12*Assumptions!D50</f>
@@ -3318,7 +3321,7 @@
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B21" s="27" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C21" s="29">
         <f>Assumptions!D52</f>
@@ -3343,7 +3346,7 @@
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B22" s="30" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C22" s="31">
         <f>C18+C19+C20+C21</f>
@@ -3394,7 +3397,7 @@
   <sheetData>
     <row r="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B1" s="13" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C1" s="13"/>
       <c r="D1" s="13"/>
@@ -3405,24 +3408,24 @@
     <row r="3" ht="24" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3" s="25"/>
       <c r="C3" s="26" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D3" s="26" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E3" s="26" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F3" s="26" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G3" s="26" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" s="27" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C5" s="28">
         <f>Drivers!C4</f>
@@ -3447,7 +3450,7 @@
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" s="27" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C6" s="29" t="str">
         <f>Drivers!C6</f>
@@ -3472,7 +3475,7 @@
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B7" s="27" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C7" s="29">
         <f>Drivers!C7</f>
@@ -3497,7 +3500,7 @@
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B8" s="27" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C8" s="29">
         <f>Drivers!C8</f>
@@ -3522,7 +3525,7 @@
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B9" s="27" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C9" s="29">
         <f>Drivers!C9</f>
@@ -3547,7 +3550,7 @@
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B10" s="30" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C10" s="31">
         <f>Drivers!C10</f>
@@ -3572,7 +3575,7 @@
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B12" s="27" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C12" s="29">
         <f>Drivers!C16</f>
@@ -3597,7 +3600,7 @@
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B13" s="27" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C13" s="29">
         <f>Drivers!C22</f>
@@ -3622,7 +3625,7 @@
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B15" s="30" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C15" s="31">
         <f>C12+C13</f>
@@ -3647,7 +3650,7 @@
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B16" s="30" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C16" s="32">
         <f>C10-C15</f>
@@ -3672,7 +3675,7 @@
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="27" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C17" s="34">
         <f>IF(C10&gt;0,C16/C10,0)</f>
@@ -3723,7 +3726,7 @@
   <sheetData>
     <row r="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B1" s="13" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C1" s="13"/>
       <c r="D1" s="13"/>
@@ -3734,24 +3737,24 @@
     <row r="3" ht="24" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3" s="25"/>
       <c r="C3" s="26" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D3" s="26" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E3" s="26" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F3" s="26" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G3" s="26" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B4" s="27" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C4" s="29">
         <f>'5-Year P&amp;L'!C16</f>
@@ -3776,7 +3779,7 @@
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" s="27" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C6" s="29">
         <f>Assumptions!D58</f>
@@ -3801,7 +3804,7 @@
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B7" s="27" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C7" s="29">
         <f>IF(Assumptions!D59&gt;0,PMT(Assumptions!D60/12,Assumptions!D61*12,-Assumptions!D59)*12,0)</f>
@@ -3826,7 +3829,7 @@
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B8" s="30" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C8" s="31">
         <f>C6+C7</f>
@@ -3851,7 +3854,7 @@
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B10" s="30" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C10" s="35">
         <f>IF(C8&gt;0,C4/C8,IF(C4&gt;0,99.9,0))</f>
@@ -3876,7 +3879,7 @@
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B12" s="27" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C12" s="29">
         <f>C4-C8</f>
@@ -3901,7 +3904,7 @@
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B14" s="30" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C14" s="37">
         <f>Assumptions!D57+C12</f>
@@ -3952,7 +3955,7 @@
   <sheetData>
     <row r="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B1" s="13" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C1" s="13"/>
       <c r="D1" s="13"/>
@@ -3963,24 +3966,24 @@
     <row r="3" ht="24" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3" s="25"/>
       <c r="C3" s="26" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D3" s="26" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E3" s="26" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F3" s="26" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G3" s="26" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B4" s="27" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C4" s="28">
         <f>Drivers!C12</f>
@@ -4005,7 +4008,7 @@
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" s="27" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C5" s="28">
         <f>Assumptions!D35</f>
@@ -4030,7 +4033,7 @@
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" s="30" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C6" s="38">
         <f>C4+C5</f>
@@ -4081,13 +4084,13 @@
   <sheetData>
     <row r="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B1" s="13" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C1" s="13"/>
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B3" s="27" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C3" s="29">
         <f>Assumptions!D59</f>
@@ -4096,7 +4099,7 @@
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B4" s="27" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C4" s="34">
         <f>Assumptions!D60</f>
@@ -4105,7 +4108,7 @@
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B5" s="27" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C5" s="28">
         <f>Assumptions!D61</f>
@@ -4114,7 +4117,7 @@
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B6" s="27" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C6" s="39">
         <f>IF(Assumptions!D59&gt;0,PMT(Assumptions!D60/12,Assumptions!D61*12,-Assumptions!D59)*12,0)</f>
@@ -4123,7 +4126,7 @@
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B8" s="27" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C8" s="35">
         <f>'Cash Flow &amp; DSCR'!C10</f>
@@ -4158,13 +4161,13 @@
   <sheetData>
     <row r="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B1" s="13" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C1" s="13"/>
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B3" s="27" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C3" s="27" t="str">
         <f>Assumptions!D5</f>
@@ -4173,7 +4176,7 @@
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B4" s="27" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C4" s="27" t="str">
         <f>Assumptions!D7</f>
@@ -4182,7 +4185,7 @@
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B5" s="27" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C5" s="27" t="str">
         <f>Assumptions!D6</f>
@@ -4191,7 +4194,7 @@
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B6" s="27" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C6" s="27">
         <f>Assumptions!D8</f>
@@ -4200,7 +4203,7 @@
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B8" s="27" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C8" s="28">
         <f>Assumptions!D16</f>
@@ -4209,7 +4212,7 @@
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B9" s="27" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C9" s="29">
         <f>Drivers!G10</f>
@@ -4218,7 +4221,7 @@
     </row>
     <row r="10" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B10" s="27" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C10" s="37">
         <f>'5-Year P&amp;L'!G16</f>
@@ -4227,7 +4230,7 @@
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B12" s="12" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C12" s="12"/>
     </row>

</xml_diff>

<commit_message>
Standardize INPUT_STYLE (blue DBEAFE fill + 1E3A5F font) on Assumptions tabs across all export formats
- excel-export.ts: Replace BOLD_FONT with applyInput() for editable cells,
  applyCalc() for computed display values (tuition tiers, projection period)
- underwriting-export.ts: Remove yellow EDITABLE_FILL (FFFFFDE8) and yellow
  (FFFFFF00) fills from buildAssumptions and buildSYAssumptions; replace with
  applyInputStyle() using standard blue input palette
- lender-proforma-export.ts: Remove local inputFill/inputFont variables;
  switch to shared inputCell() helper from workbook-helpers.ts
- underwriting-workbook.ts and formula-export.ts already used inputCell() — no changes needed

All 24 QA, 3 formula-results, and 33 parity checks pass.
</commit_message>
<xml_diff>
--- a/artifacts/api-server/qa-output/Lender_Pro_Forma_Charter_ADA_Grade-Band.xlsx
+++ b/artifacts/api-server/qa-output/Lender_Pro_Forma_Charter_ADA_Grade-Band.xlsx
@@ -659,7 +659,7 @@
     <numFmt numFmtId="166" formatCode="0.0%;[Red](0.0%);&quot;-&quot;"/>
     <numFmt numFmtId="167" formatCode="0.00x"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -727,6 +727,9 @@
       <color rgb="FF1E293B"/>
       <sz val="14"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <color rgb="FF1E3A5F"/>
     </font>
     <font>
       <i/>
@@ -888,31 +891,31 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="12" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="12" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="12" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="10" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="12" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
@@ -922,57 +925,57 @@
     <xf numFmtId="165" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="17" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="16" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="17" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="16" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="17" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="166" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="16" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="17" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="16" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="17" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="16" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="17" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="17" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="16" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="17" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="16" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="17" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="16" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="17" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="16" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="17" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="16" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="17" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -981,10 +984,10 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>

</xml_diff>

<commit_message>
Replace hardcoded row offsets with dynamic tracking in lender proforma export
Updates artifacts/api-server/src/lib/lender-proforma-export.ts to use a dynamic row cursor instead of hardcoded values for various sections, improving resilience to future changes.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: a1e7a024-8deb-4e05-bb93-350fde674463
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 8b85a13c-0b97-4c45-aeec-f8c1c12dee4c
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/27fdbaf7-67db-442f-83d4-bebcb570d0b5/a1e7a024-8deb-4e05-bb93-350fde674463/1ucI1Ab
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/api-server/qa-output/Lender_Pro_Forma_Charter_ADA_Grade-Band.xlsx
+++ b/artifacts/api-server/qa-output/Lender_Pro_Forma_Charter_ADA_Grade-Band.xlsx
@@ -2620,7 +2620,7 @@
     <tabColor rgb="FFD97706"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:E78"/>
+  <dimension ref="B1:E77"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -3028,32 +3028,40 @@
         <v>10</v>
       </c>
     </row>
-    <row r="64" ht="24" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B64" s="17" t="s">
+    <row r="63" ht="24" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B63" s="17" t="s">
         <v>95</v>
       </c>
-      <c r="C64" s="17"/>
-      <c r="D64" s="17"/>
+      <c r="C63" s="17"/>
+      <c r="D63" s="17"/>
+    </row>
+    <row r="65" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C65" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="D65" s="19" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="66" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C66" s="18" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D66" s="19" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="67" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C67" s="18" t="s">
-        <v>98</v>
-      </c>
-      <c r="D67" s="19" t="s">
-        <v>99</v>
+        <v>100</v>
+      </c>
+      <c r="D67" s="20">
+        <v>0</v>
       </c>
     </row>
     <row r="68" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C68" s="18" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D68" s="20">
         <v>0</v>
@@ -3061,71 +3069,63 @@
     </row>
     <row r="69" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C69" s="18" t="s">
-        <v>101</v>
-      </c>
-      <c r="D69" s="20">
-        <v>0</v>
+        <v>102</v>
+      </c>
+      <c r="D69" s="23">
+        <v>0.95</v>
       </c>
     </row>
     <row r="70" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C70" s="18" t="s">
-        <v>102</v>
-      </c>
-      <c r="D70" s="23">
-        <v>0.95</v>
+        <v>103</v>
+      </c>
+      <c r="D70" s="21">
+        <v>8200</v>
       </c>
     </row>
     <row r="71" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C71" s="18" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D71" s="21">
-        <v>8200</v>
+        <v>9100</v>
       </c>
     </row>
     <row r="72" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C72" s="18" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D72" s="21">
-        <v>9100</v>
-      </c>
-    </row>
-    <row r="73" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C73" s="18" t="s">
-        <v>105</v>
-      </c>
-      <c r="D73" s="21">
         <v>10500</v>
       </c>
     </row>
+    <row r="74" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C74" s="24" t="s">
+        <v>106</v>
+      </c>
+      <c r="D74" s="24"/>
+    </row>
     <row r="75" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C75" s="24" t="s">
-        <v>106</v>
-      </c>
-      <c r="D75" s="24"/>
+      <c r="C75" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="D75" s="25" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="76" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C76" s="18" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D76" s="25" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="77" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C77" s="18" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D77" s="25" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="78" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C78" s="18" t="s">
-        <v>111</v>
-      </c>
-      <c r="D78" s="25" t="s">
         <v>112</v>
       </c>
     </row>
@@ -3138,8 +3138,8 @@
     <mergeCell ref="B30:D30"/>
     <mergeCell ref="B44:D44"/>
     <mergeCell ref="B55:D55"/>
-    <mergeCell ref="B64:D64"/>
-    <mergeCell ref="C75:D75"/>
+    <mergeCell ref="B63:D63"/>
+    <mergeCell ref="C74:D74"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>